<commit_message>
feat: 数值修正层 values-patch — 策划数值经Excel→patch→export, 全程不动源证据baseline
关键架构(回应用户'不改baseline'):
- baseline(multisource-baseline.json) 被 sha256 锚定(verify.js:54, data-import.test.js, validator.js:31)
  ——它是「从源仓库抽取的证据快照」, 改它=伪造源证据, 触发 'Baseline SHA-256 changed' 失败。
- 新增 data/runtime/values-patch.json 修正层: 承接所有策划数值改动(装备等级/怪物名/掉率/价格),
  只叠加、不改 baseline。

本次落地:
- export-numbers-xlsx: 从 baseline+patch 合并导出 Excel(反映当前生效值); 支持 equipment.level→required_level,
  monster_definitions.display_name→怪名 的映射。
- import-numbers-xlsx: 改为对比 Excel 与基线差异→生成 values-patch.json(而非改 baseline); --dry-run 预览。
- export-task1-content: 新增 applyValuesPatch, 导出时对 monsters/gameplay(equipment/drop_relations...)做字段覆盖;
  装备 level→required_level 映射。
- 已跑通完整闭环: 改Excel(怪名+装备等级)→import生成patch→export→游戏内容验证(沙漠蝎王/战铠140/皇冠125)。
- 测试 195/195 通过; verify.js --core 13/13 含 'baseline byte hash' pass(证明未碰baseline)。
</commit_message>
<xml_diff>
--- a/design/numbers/gameplay-numbers.xlsx
+++ b/design/numbers/gameplay-numbers.xlsx
@@ -5396,7 +5396,7 @@
         <v>entity.monster.cbe1f18ad64d8183</v>
       </c>
       <c r="B250" t="str">
-        <v>你看到:</v>
+        <v>沙漠蝎王</v>
       </c>
       <c r="C250">
         <v>124</v>
@@ -5736,7 +5736,7 @@
         <v>entity.monster.ee31f5f9df972310</v>
       </c>
       <c r="B267" t="str">
-        <v>你看到:</v>
+        <v>吞兽</v>
       </c>
       <c r="C267">
         <v>118</v>
@@ -5756,7 +5756,7 @@
         <v>entity.monster.e9a94e35bb84c0dd</v>
       </c>
       <c r="B268" t="str">
-        <v>你看到:</v>
+        <v>落日蛮牛</v>
       </c>
       <c r="C268">
         <v>54</v>
@@ -63739,8 +63739,8 @@
       <c r="C29" t="str">
         <v>+天魔荆棘皇冠</v>
       </c>
-      <c r="D29" t="str">
-        <v/>
+      <c r="D29">
+        <v>125</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -63768,8 +63768,8 @@
       <c r="C30" t="str">
         <v>+天魔玄夜战铠</v>
       </c>
-      <c r="D30" t="str">
-        <v/>
+      <c r="D30">
+        <v>140</v>
       </c>
       <c r="E30" t="str">
         <v/>

</xml_diff>